<commit_message>
test: simulate fresh month (workbook through April)
</commit_message>
<xml_diff>
--- a/mw-historic-data.xlsx
+++ b/mw-historic-data.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P198"/>
+  <dimension ref="A1:P197"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -10672,62 +10672,6 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="D198" s="23" t="n">
-        <v>6583</v>
-      </c>
-      <c r="E198" s="24" t="n">
-        <v>7041836263</v>
-      </c>
-      <c r="F198" s="24" t="n">
-        <v>1069700</v>
-      </c>
-      <c r="G198" s="25">
-        <f>IFERROR(F198/F186-1,"")</f>
-        <v/>
-      </c>
-      <c r="H198" s="24" t="n">
-        <v>910000</v>
-      </c>
-      <c r="I198" s="23" t="n">
-        <v>17698</v>
-      </c>
-      <c r="J198" s="23" t="n">
-        <v>26927</v>
-      </c>
-      <c r="K198" s="25" t="n">
-        <v>0.357</v>
-      </c>
-      <c r="L198" s="26">
-        <f>J198/D198</f>
-        <v/>
-      </c>
-      <c r="M198" s="26" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="N198" s="27" t="n">
-        <v>27</v>
-      </c>
-      <c r="O198" s="27" t="n">
-        <v>42</v>
-      </c>
-      <c r="P198" s="25" t="n">
-        <v>0.98</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -10741,7 +10685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P198"/>
+  <dimension ref="A1:P197"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -20983,62 +20927,6 @@
         <v>0.979</v>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="D198" s="23" t="n">
-        <v>1183</v>
-      </c>
-      <c r="E198" s="24" t="n">
-        <v>1392781792</v>
-      </c>
-      <c r="F198" s="24" t="n">
-        <v>1177330</v>
-      </c>
-      <c r="G198" s="25">
-        <f>IFERROR(F198/F186-1,"")</f>
-        <v/>
-      </c>
-      <c r="H198" s="24" t="n">
-        <v>1090000</v>
-      </c>
-      <c r="I198" s="23" t="n">
-        <v>3323</v>
-      </c>
-      <c r="J198" s="23" t="n">
-        <v>5252</v>
-      </c>
-      <c r="K198" s="25" t="n">
-        <v>0.339</v>
-      </c>
-      <c r="L198" s="26">
-        <f>J198/D198</f>
-        <v/>
-      </c>
-      <c r="M198" s="26" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="N198" s="27" t="n">
-        <v>28</v>
-      </c>
-      <c r="O198" s="27" t="n">
-        <v>42</v>
-      </c>
-      <c r="P198" s="25" t="n">
-        <v>0.98</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -21052,7 +20940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P198"/>
+  <dimension ref="A1:P197"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -31294,62 +31182,6 @@
         <v>0.988</v>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="D198" s="23" t="n">
-        <v>2377</v>
-      </c>
-      <c r="E198" s="24" t="n">
-        <v>2634409008</v>
-      </c>
-      <c r="F198" s="24" t="n">
-        <v>1108292</v>
-      </c>
-      <c r="G198" s="25">
-        <f>IFERROR(F198/F186-1,"")</f>
-        <v/>
-      </c>
-      <c r="H198" s="24" t="n">
-        <v>885000</v>
-      </c>
-      <c r="I198" s="23" t="n">
-        <v>6401</v>
-      </c>
-      <c r="J198" s="23" t="n">
-        <v>9916</v>
-      </c>
-      <c r="K198" s="25" t="n">
-        <v>0.366</v>
-      </c>
-      <c r="L198" s="26">
-        <f>J198/D198</f>
-        <v/>
-      </c>
-      <c r="M198" s="26" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="N198" s="27" t="n">
-        <v>26</v>
-      </c>
-      <c r="O198" s="27" t="n">
-        <v>40</v>
-      </c>
-      <c r="P198" s="25" t="n">
-        <v>0.99</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -31363,7 +31195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P198"/>
+  <dimension ref="A1:P197"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -41605,62 +41437,6 @@
         <v>0.969</v>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="D198" s="23" t="n">
-        <v>247</v>
-      </c>
-      <c r="E198" s="24" t="n">
-        <v>216306128</v>
-      </c>
-      <c r="F198" s="24" t="n">
-        <v>875733</v>
-      </c>
-      <c r="G198" s="25">
-        <f>IFERROR(F198/F186-1,"")</f>
-        <v/>
-      </c>
-      <c r="H198" s="24" t="n">
-        <v>815000</v>
-      </c>
-      <c r="I198" s="23" t="n">
-        <v>657</v>
-      </c>
-      <c r="J198" s="23" t="n">
-        <v>1122</v>
-      </c>
-      <c r="K198" s="25" t="n">
-        <v>0.307</v>
-      </c>
-      <c r="L198" s="26">
-        <f>J198/D198</f>
-        <v/>
-      </c>
-      <c r="M198" s="26" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="N198" s="27" t="n">
-        <v>34</v>
-      </c>
-      <c r="O198" s="27" t="n">
-        <v>49</v>
-      </c>
-      <c r="P198" s="25" t="n">
-        <v>0.96</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -41674,7 +41450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P198"/>
+  <dimension ref="A1:P197"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -51916,62 +51692,6 @@
         <v>0.973</v>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="D198" s="23" t="n">
-        <v>1106</v>
-      </c>
-      <c r="E198" s="24" t="n">
-        <v>1057356568</v>
-      </c>
-      <c r="F198" s="24" t="n">
-        <v>956019</v>
-      </c>
-      <c r="G198" s="25">
-        <f>IFERROR(F198/F186-1,"")</f>
-        <v/>
-      </c>
-      <c r="H198" s="24" t="n">
-        <v>875000</v>
-      </c>
-      <c r="I198" s="23" t="n">
-        <v>3267</v>
-      </c>
-      <c r="J198" s="23" t="n">
-        <v>5053</v>
-      </c>
-      <c r="K198" s="25" t="n">
-        <v>0.324</v>
-      </c>
-      <c r="L198" s="26">
-        <f>J198/D198</f>
-        <v/>
-      </c>
-      <c r="M198" s="26" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="N198" s="27" t="n">
-        <v>29</v>
-      </c>
-      <c r="O198" s="27" t="n">
-        <v>44</v>
-      </c>
-      <c r="P198" s="25" t="n">
-        <v>0.98</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -51985,7 +51705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P198"/>
+  <dimension ref="A1:P197"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -62227,62 +61947,6 @@
         <v>0.961</v>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="D198" s="23" t="n">
-        <v>816</v>
-      </c>
-      <c r="E198" s="24" t="n">
-        <v>1018593994</v>
-      </c>
-      <c r="F198" s="24" t="n">
-        <v>1248277</v>
-      </c>
-      <c r="G198" s="25">
-        <f>IFERROR(F198/F186-1,"")</f>
-        <v/>
-      </c>
-      <c r="H198" s="24" t="n">
-        <v>1050000</v>
-      </c>
-      <c r="I198" s="23" t="n">
-        <v>1969</v>
-      </c>
-      <c r="J198" s="23" t="n">
-        <v>2870</v>
-      </c>
-      <c r="K198" s="25" t="n">
-        <v>0.381</v>
-      </c>
-      <c r="L198" s="26">
-        <f>J198/D198</f>
-        <v/>
-      </c>
-      <c r="M198" s="26" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="N198" s="27" t="n">
-        <v>29</v>
-      </c>
-      <c r="O198" s="27" t="n">
-        <v>44</v>
-      </c>
-      <c r="P198" s="25" t="n">
-        <v>0.97</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -62296,7 +61960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P198"/>
+  <dimension ref="A1:P197"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -72538,62 +72202,6 @@
         <v>0.993</v>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="D198" s="23" t="n">
-        <v>804</v>
-      </c>
-      <c r="E198" s="24" t="n">
-        <v>684255873</v>
-      </c>
-      <c r="F198" s="24" t="n">
-        <v>851065</v>
-      </c>
-      <c r="G198" s="25">
-        <f>IFERROR(F198/F186-1,"")</f>
-        <v/>
-      </c>
-      <c r="H198" s="24" t="n">
-        <v>801000</v>
-      </c>
-      <c r="I198" s="23" t="n">
-        <v>1978</v>
-      </c>
-      <c r="J198" s="23" t="n">
-        <v>2563</v>
-      </c>
-      <c r="K198" s="25" t="n">
-        <v>0.404</v>
-      </c>
-      <c r="L198" s="26">
-        <f>J198/D198</f>
-        <v/>
-      </c>
-      <c r="M198" s="26" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="N198" s="27" t="n">
-        <v>24</v>
-      </c>
-      <c r="O198" s="27" t="n">
-        <v>37</v>
-      </c>
-      <c r="P198" s="25" t="n">
-        <v>0.99</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -72607,7 +72215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P198"/>
+  <dimension ref="A1:P197"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -82849,62 +82457,6 @@
         <v>0.971</v>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>May</t>
-        </is>
-      </c>
-      <c r="D198" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="E198" s="24" t="n">
-        <v>38132900</v>
-      </c>
-      <c r="F198" s="24" t="n">
-        <v>762658</v>
-      </c>
-      <c r="G198" s="25">
-        <f>IFERROR(F198/F186-1,"")</f>
-        <v/>
-      </c>
-      <c r="H198" s="24" t="n">
-        <v>733000</v>
-      </c>
-      <c r="I198" s="23" t="n">
-        <v>103</v>
-      </c>
-      <c r="J198" s="23" t="n">
-        <v>151</v>
-      </c>
-      <c r="K198" s="25" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="L198" s="26">
-        <f>J198/D198</f>
-        <v/>
-      </c>
-      <c r="M198" s="26" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="N198" s="27" t="n">
-        <v>33</v>
-      </c>
-      <c r="O198" s="27" t="n">
-        <v>41</v>
-      </c>
-      <c r="P198" s="25" t="n">
-        <v>0.97</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>